<commit_message>
Add Pathway and Causeway Tier A USC recruiter matches
Expand verified buy-side list with Jodi M. Field (Pathway Capital HR/talent
acquisition) and Jaime Rochon (Causeway Capital HR/recruiting), both with USC
ties on official firm pages. Sync missing Tier B CSV rows and regenerate Excel
workbooks.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Recruiters/Tier_A_1_to_10B_AUM.xlsx
+++ b/Recruiters/Tier_A_1_to_10B_AUM.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Tier A 1-10B AUM" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Recruiters" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,6 +28,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="3">
@@ -40,7 +44,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
-        <bgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
   </fills>
@@ -56,9 +59,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -426,19 +435,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="55" customWidth="1" min="8" max="8"/>
-    <col width="45" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -449,155 +457,144 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>AUM_Bucket</t>
+          <t>Firm</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Firm</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>AUM (approx.)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>AUM_Approx</t>
+          <t>Named Contact</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Named_Contact</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Role</t>
+          <t>USC Connection</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>USC_Connection</t>
+          <t>Official Source URL</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Official_Source_URL</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>$1-10B</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Gryphon Investors</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Private Equity</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>~$7B</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>7B</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Barry Becker</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Managing Director, Human Resources team</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>MBA specializing in Human Resources, University of Southern California</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>https://www.gryphon-inv.com/team/barry-becker/</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Operations Resources Group; portfolio company HR/talent initiatives</t>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>$1-10B AUM focus; portfolio HR/talent initiatives</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>$1-10B</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>JMI Equity</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Growth Equity / Software PE</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>~$6B</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>6B</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Haley Donzella</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>HR Manager</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Master's in Human Resource Management, University of Southern California</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>https://www.jmi.com/team/donzella-haley/</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Internal talent, professional development, performance management</t>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>$1-10B AUM focus; internal talent programs</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>